<commit_message>
Updated CDE ID workflow for more accurate mapping
</commit_message>
<xml_diff>
--- a/CDE_ID_detective_revamp/in/Testfile.xlsx
+++ b/CDE_ID_detective_revamp/in/Testfile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmaefos\Code Stuffs\CDE_detective\CDE_ID_detective_revamp\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A45D79-AD2C-43B2-9762-8753FB6771C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9041BD5D-201C-41D4-A753-1309F3A61AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30750" yWindow="7230" windowWidth="25830" windowHeight="15105" xr2:uid="{B4172F7E-1829-43FF-A6F3-7109D1C548C2}"/>
+    <workbookView xWindow="-38520" yWindow="4380" windowWidth="38640" windowHeight="21120" xr2:uid="{B4172F7E-1829-43FF-A6F3-7109D1C548C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -161,42 +161,21 @@
     <t>0|1|2|3|4|5|6|7|8|9|10</t>
   </si>
   <si>
-    <t>bpisev</t>
-  </si>
-  <si>
-    <t>BPIWrstPnLast24HRtngScl</t>
-  </si>
-  <si>
     <t>Worst Pain in the Last 24 Hours</t>
   </si>
   <si>
     <t>0=No pain (0)|1=1|2=2|3=3|4=4|5=5|6=6|7=7|8=8|9=9|10=Pain as bad as you can imagine (10)</t>
   </si>
   <si>
-    <t>BPILeastPnLst24HRtngScl</t>
-  </si>
-  <si>
     <t>Least Pain in the Last 24 Hours</t>
   </si>
   <si>
-    <t>BPIAvgPainRtngScl</t>
-  </si>
-  <si>
     <t>Average Pain</t>
   </si>
   <si>
-    <t>BPICurrentPainRtngScl</t>
-  </si>
-  <si>
     <t>Current Pain</t>
   </si>
   <si>
-    <t>gad7</t>
-  </si>
-  <si>
-    <t>GAD2FeelNervScl</t>
-  </si>
-  <si>
     <t>Feeling Nervous</t>
   </si>
   <si>
@@ -206,47 +185,68 @@
     <t>0=Not at all|1=Several Days|2=More than half the days|3=Nearly every day</t>
   </si>
   <si>
-    <t>GAD2NotStopWryScl</t>
-  </si>
-  <si>
     <t>Unable to Stop Worrying</t>
   </si>
   <si>
-    <t>GAD7WryTooMchScl</t>
-  </si>
-  <si>
     <t>Worrying Too Much</t>
   </si>
   <si>
-    <t>GAD7TroubRelxScl</t>
-  </si>
-  <si>
     <t>Trouble Relaxing</t>
   </si>
   <si>
-    <t>GAD7RstlessScl</t>
-  </si>
-  <si>
     <t>Being Restless</t>
   </si>
   <si>
-    <t>GAD7EasyAnnoyedScl</t>
-  </si>
-  <si>
     <t>Becoming Easily Annoyed/Irritable</t>
   </si>
   <si>
-    <t>GAD7FeelAfrdScl</t>
-  </si>
-  <si>
     <t>Feeling Afraid</t>
+  </si>
+  <si>
+    <t>FORM1</t>
+  </si>
+  <si>
+    <t>FORM2</t>
+  </si>
+  <si>
+    <t>AvgPainRtngScl</t>
+  </si>
+  <si>
+    <t>CurrentPainRtngScl</t>
+  </si>
+  <si>
+    <t>LeastPnLst24HRtngScl</t>
+  </si>
+  <si>
+    <t>WrstPnLast24HRtngScl</t>
+  </si>
+  <si>
+    <t>FeelNervScl</t>
+  </si>
+  <si>
+    <t>NotStopWryScl</t>
+  </si>
+  <si>
+    <t>EasyAnnoyedScl</t>
+  </si>
+  <si>
+    <t>FeelAfrdScl</t>
+  </si>
+  <si>
+    <t>RstlessScl</t>
+  </si>
+  <si>
+    <t>TroubRelxScl</t>
+  </si>
+  <si>
+    <t>WryTooMchScl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -377,6 +377,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1104,6 +1110,7 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="33.19921875" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.45">
@@ -1263,16 +1270,16 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
         <v>31</v>
@@ -1281,7 +1288,7 @@
         <v>40</v>
       </c>
       <c r="N5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.45">
@@ -1289,16 +1296,16 @@
         <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F6" t="s">
         <v>31</v>
@@ -1307,7 +1314,7 @@
         <v>40</v>
       </c>
       <c r="N6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.45">
@@ -1315,16 +1322,16 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
         <v>31</v>
@@ -1333,7 +1340,7 @@
         <v>40</v>
       </c>
       <c r="N7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.45">
@@ -1341,16 +1348,16 @@
         <v>30</v>
       </c>
       <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" t="s">
         <v>41</v>
       </c>
-      <c r="C8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" t="s">
-        <v>43</v>
-      </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F8" t="s">
         <v>31</v>
@@ -1359,7 +1366,7 @@
         <v>40</v>
       </c>
       <c r="N8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.45">
@@ -1367,25 +1374,25 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F9" t="s">
         <v>31</v>
       </c>
       <c r="J9" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N9" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.45">
@@ -1393,25 +1400,25 @@
         <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="F10" t="s">
         <v>31</v>
       </c>
       <c r="J10" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N10" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.45">
@@ -1419,25 +1426,25 @@
         <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
         <v>31</v>
       </c>
       <c r="J11" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N11" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.45">
@@ -1445,25 +1452,25 @@
         <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="F12" t="s">
         <v>31</v>
       </c>
       <c r="J12" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N12" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.45">
@@ -1471,25 +1478,25 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="F13" t="s">
         <v>31</v>
       </c>
       <c r="J13" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N13" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.45">
@@ -1497,25 +1504,25 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" t="s">
         <v>51</v>
       </c>
-      <c r="C14" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" t="s">
-        <v>61</v>
-      </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F14" t="s">
         <v>31</v>
       </c>
       <c r="J14" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N14" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.45">
@@ -1523,25 +1530,25 @@
         <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F15" t="s">
         <v>31</v>
       </c>
       <c r="J15" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N15" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1550,6 +1557,7 @@
       <sortCondition ref="B1:B15"/>
     </sortState>
   </autoFilter>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated script and cleaned folders
</commit_message>
<xml_diff>
--- a/CDE_ID_detective_revamp/in/Testfile.xlsx
+++ b/CDE_ID_detective_revamp/in/Testfile.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmaefos\Code Stuffs\CDE_detective\CDE_ID_detective_revamp\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9041BD5D-201C-41D4-A753-1309F3A61AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817B149D-0F69-43F3-8A18-7056A50B2854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="4380" windowWidth="38640" windowHeight="21120" xr2:uid="{B4172F7E-1829-43FF-A6F3-7109D1C548C2}"/>
+    <workbookView xWindow="-19305" yWindow="4500" windowWidth="19410" windowHeight="20985" xr2:uid="{B4172F7E-1829-43FF-A6F3-7109D1C548C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AD$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AC$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="68">
-  <si>
-    <t>schemaVersion</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="172">
   <si>
     <t>section</t>
   </si>
@@ -128,9 +125,6 @@
     <t>relatedConcepts[0].id</t>
   </si>
   <si>
-    <t>0.3.2</t>
-  </si>
-  <si>
     <t>integer</t>
   </si>
   <si>
@@ -240,6 +234,324 @@
   </si>
   <si>
     <t>WryTooMchScl</t>
+  </si>
+  <si>
+    <t>FORM3</t>
+  </si>
+  <si>
+    <t>subject_id</t>
+  </si>
+  <si>
+    <t>visit</t>
+  </si>
+  <si>
+    <t>tobaccoproductscl</t>
+  </si>
+  <si>
+    <t>alcoholusemalescl</t>
+  </si>
+  <si>
+    <t>alcoholusefemalescl</t>
+  </si>
+  <si>
+    <t>drugusescl</t>
+  </si>
+  <si>
+    <t>prescriptionmedusescl</t>
+  </si>
+  <si>
+    <t>overallyn</t>
+  </si>
+  <si>
+    <t>Subject ID</t>
+  </si>
+  <si>
+    <t>Study Visit</t>
+  </si>
+  <si>
+    <t>have you used any tobacco product (for example, cigarettes, e-cigarettes, cigars, pipes, or smokeless tobacco)?</t>
+  </si>
+  <si>
+    <t>how often have you had 5 or more drinks containing alcohol in one day? One standard drink is about 1 small glass of wine (5 oz), 1 beer (12 oz), or 1 single shot of liquor.</t>
+  </si>
+  <si>
+    <t>how often have you had 4 or more drinks containing alcohol in one day? One standard drink is about 1 small glass of wine (5 oz), 1 beer (12 oz), or 1 single shot of liquor.</t>
+  </si>
+  <si>
+    <t>have you used any drugs including marijuana, cocaine or crack,heroin, methamphetamine (crystal meth), hallucinogens, ecstasy/MDMA?</t>
+  </si>
+  <si>
+    <t>have you used any prescription medications just for the feeling, more than prescribed or that were not prescribed for you? Prescription medications that may be used this way include: Opiate pain relievers (for example, OxyContin, Vicodin, Percocet, Methadone) Medications for anxiety or sleeping (for example, Xanax, Ativan, Klonopin) Medications for ADHD (for example, Adderall or Ritalin)?</t>
+  </si>
+  <si>
+    <t>Overall TAPS part 1</t>
+  </si>
+  <si>
+    <t>1,Visit 1 | 2,Visit 2</t>
+  </si>
+  <si>
+    <t>0,Daily or Almost Daily | 1,Weekly | 2,Monthly | 3,Less Than Monthly | 4,Never</t>
+  </si>
+  <si>
+    <t>sum([tapstobaccoproductscl], [tapsalcoholusemalescl], [tapsalcoholusefemalescl], [tapsdrugusescl], [tapsprescriptionmedusescl] &gt; 1, 1, 0)</t>
+  </si>
+  <si>
+    <t>brthdtc</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>sex</t>
+  </si>
+  <si>
+    <t>genident</t>
+  </si>
+  <si>
+    <t>ethnic</t>
+  </si>
+  <si>
+    <t>race___1</t>
+  </si>
+  <si>
+    <t>race___2</t>
+  </si>
+  <si>
+    <t>race___3</t>
+  </si>
+  <si>
+    <t>race___4</t>
+  </si>
+  <si>
+    <t>race___5</t>
+  </si>
+  <si>
+    <t>race___6</t>
+  </si>
+  <si>
+    <t>race___7</t>
+  </si>
+  <si>
+    <t>edlevel</t>
+  </si>
+  <si>
+    <t>empstat</t>
+  </si>
+  <si>
+    <t>maristat</t>
+  </si>
+  <si>
+    <t>hhnum</t>
+  </si>
+  <si>
+    <t>paindur</t>
+  </si>
+  <si>
+    <t>baseline_demographics</t>
+  </si>
+  <si>
+    <t>Date of Birth: (mm/dd/yyyy)</t>
+  </si>
+  <si>
+    <t>Age:</t>
+  </si>
+  <si>
+    <t>Sex at birth:</t>
+  </si>
+  <si>
+    <t>Gender Identity:</t>
+  </si>
+  <si>
+    <t>Ethnicity: (Choose one)</t>
+  </si>
+  <si>
+    <t>Race: American Indian or Alaskan Native</t>
+  </si>
+  <si>
+    <t>Race: Asian</t>
+  </si>
+  <si>
+    <t>Race: Black or African American</t>
+  </si>
+  <si>
+    <t>Race: Native Hawaiian or Pacific Islander</t>
+  </si>
+  <si>
+    <t>Race: White</t>
+  </si>
+  <si>
+    <t>Race: Unknown</t>
+  </si>
+  <si>
+    <t>Race: Not reported</t>
+  </si>
+  <si>
+    <t>What is the highest level of education you have completed?</t>
+  </si>
+  <si>
+    <t>What is your current employment status?</t>
+  </si>
+  <si>
+    <t>What category best describes your current relationship status?</t>
+  </si>
+  <si>
+    <t>Including yourself, how many people live in your household?</t>
+  </si>
+  <si>
+    <t>How long have you had the type of pain for which you are enrolled in this study? (Please list the number of months)</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Date of Birth: (mm/dd/yyyy)</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Age:</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Sex at birth:</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Gender Identity:</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Ethnicity: (Choose one)</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Race: (Choose all that apply)[choice=American Indian or Alaskan Native]</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Race: (Choose all that apply)[choice=Asian]</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Race: (Choose all that apply)[choice=Black or African American]</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Race: (Choose all that apply)[choice=Native Hawaiian or Pacific Islander]</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Race: (Choose all that apply)[choice=White]</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Race: (Choose all that apply)[choice=Unknown]</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Race: (Choose all that apply)[choice=Not reported]</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: What is the highest level of education you have completed?</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: What is your current employment status?</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: What category best describes your current relationship status?</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: Including yourself, how many people live in your household?</t>
+  </si>
+  <si>
+    <t>Part of the Minimal Dataset: How long have you had the type of pain for which you are enrolled in this study? (Please list the number of months)</t>
+  </si>
+  <si>
+    <t>1|2|3|4</t>
+  </si>
+  <si>
+    <t>0|1</t>
+  </si>
+  <si>
+    <t>1|2|3|4|5|6|7|8|9</t>
+  </si>
+  <si>
+    <t>1|2|3|4|5</t>
+  </si>
+  <si>
+    <t>1=Male|2=Female|3=Unknown|4=Intersex</t>
+  </si>
+  <si>
+    <t>1=Male|2=Female|3=Unknown|4=Other, specify, [Open Text]</t>
+  </si>
+  <si>
+    <t>1=Hispanic or Latino|2=Not Hispanic or Latino|3=Unknown|4=Not reported</t>
+  </si>
+  <si>
+    <t>0=Unchecked|1=Checked</t>
+  </si>
+  <si>
+    <t>1=Primary (Elementary School)|2=Lower Secondary (Middle School)|3=Upper Secondary (High School)|4=Diploma or equivalent (GED)|5=Some college/Certificate|6=Vocation/Trade School|7=Bachelor’s Degree|8=Some Graduate or Professional School|9=Graduate or Professional School diploma</t>
+  </si>
+  <si>
+    <t>1=Full-time employment|2=Not employed|3=Part-time employment|4=Retired</t>
+  </si>
+  <si>
+    <t>1=Divorced|2=Married|3=Never married|4=Separated|5=Widowed</t>
+  </si>
+  <si>
+    <t>fibromyalgia_fm_survey_criteria_2016</t>
+  </si>
+  <si>
+    <t>face</t>
+  </si>
+  <si>
+    <t>Face</t>
+  </si>
+  <si>
+    <t>Widespread Pain Index (WPI) and Symptom Severity Index (SSI): Face</t>
+  </si>
+  <si>
+    <t>rt_jaw</t>
+  </si>
+  <si>
+    <t>Rt Jaw</t>
+  </si>
+  <si>
+    <t>Widespread Pain Index (WPI) and Symptom Severity Index (SSI): Rt Jaw</t>
+  </si>
+  <si>
+    <t>lt_jaw</t>
+  </si>
+  <si>
+    <t>Lt Jaw</t>
+  </si>
+  <si>
+    <t>Widespread Pain Index (WPI) and Symptom Severity Index (SSI): Lt Jaw</t>
+  </si>
+  <si>
+    <t>rt_breast</t>
+  </si>
+  <si>
+    <t>Rt Breast</t>
+  </si>
+  <si>
+    <t>Widespread Pain Index (WPI) and Symptom Severity Index (SSI): Rt Breast</t>
+  </si>
+  <si>
+    <t>lt_breast</t>
+  </si>
+  <si>
+    <t>Lt Breast</t>
+  </si>
+  <si>
+    <t>Widespread Pain Index (WPI) and Symptom Severity Index (SSI): Lt Breast</t>
+  </si>
+  <si>
+    <t>rt_upper_arm</t>
+  </si>
+  <si>
+    <t>Rt upper arm</t>
+  </si>
+  <si>
+    <t>Widespread Pain Index (WPI) and Symptom Severity Index (SSI): Rt upper arm</t>
+  </si>
+  <si>
+    <t>lt_upper_arm</t>
+  </si>
+  <si>
+    <t>Lt upper arm</t>
+  </si>
+  <si>
+    <t>Widespread Pain Index (WPI) and Symptom Severity Index (SSI): Lt upper arm</t>
+  </si>
+  <si>
+    <t>1=Yes|0=No</t>
   </si>
 </sst>
 </file>
@@ -1106,14 +1418,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4F619F0-927D-42BE-B802-34E76A1D5A02}">
-  <dimension ref="A1:AD15"/>
+  <dimension ref="A1:AC47"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="33.19921875" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="1" max="1" width="33.19921875" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1201,360 +1513,859 @@
       <c r="AC1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.45">
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
         <v>30</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
         <v>33</v>
       </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
         <v>30</v>
       </c>
-      <c r="B3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.45">
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
         <v>55</v>
       </c>
       <c r="C5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="M5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" t="s">
         <v>57</v>
       </c>
-      <c r="D5" t="s">
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" t="s">
+        <v>38</v>
+      </c>
+      <c r="M8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
         <v>44</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D9" t="s">
         <v>44</v>
       </c>
-      <c r="F5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" t="s">
-        <v>40</v>
-      </c>
-      <c r="N5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" t="s">
         <v>45</v>
       </c>
-      <c r="E6" t="s">
+      <c r="M9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="I10" t="s">
         <v>45</v>
       </c>
-      <c r="F6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J6" t="s">
-        <v>40</v>
-      </c>
-      <c r="N6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" t="s">
-        <v>55</v>
-      </c>
-      <c r="C7" t="s">
-        <v>59</v>
-      </c>
-      <c r="D7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" t="s">
-        <v>31</v>
-      </c>
-      <c r="J7" t="s">
-        <v>40</v>
-      </c>
-      <c r="N7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" t="s">
-        <v>31</v>
-      </c>
-      <c r="J8" t="s">
-        <v>40</v>
-      </c>
-      <c r="N8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="M10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" t="s">
         <v>61</v>
       </c>
-      <c r="D9" t="s">
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" t="s">
+        <v>29</v>
+      </c>
+      <c r="I11" t="s">
+        <v>45</v>
+      </c>
+      <c r="M11" t="s">
         <v>46</v>
       </c>
-      <c r="E9" t="s">
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" t="s">
+        <v>29</v>
+      </c>
+      <c r="I12" t="s">
+        <v>45</v>
+      </c>
+      <c r="M12" t="s">
         <v>46</v>
       </c>
-      <c r="F9" t="s">
-        <v>31</v>
-      </c>
-      <c r="J9" t="s">
-        <v>47</v>
-      </c>
-      <c r="N9" t="s">
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>29</v>
+      </c>
+      <c r="I13" t="s">
+        <v>45</v>
+      </c>
+      <c r="M13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" t="s">
+        <v>45</v>
+      </c>
+      <c r="M14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" t="s">
-        <v>62</v>
-      </c>
-      <c r="D10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" t="s">
-        <v>49</v>
-      </c>
-      <c r="F10" t="s">
-        <v>31</v>
-      </c>
-      <c r="J10" t="s">
-        <v>47</v>
-      </c>
-      <c r="N10" t="s">
+      <c r="D15" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" t="s">
-        <v>31</v>
-      </c>
-      <c r="J11" t="s">
-        <v>47</v>
-      </c>
-      <c r="N11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" t="s">
-        <v>31</v>
-      </c>
-      <c r="J12" t="s">
-        <v>47</v>
-      </c>
-      <c r="N12" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" t="s">
-        <v>65</v>
-      </c>
-      <c r="D13" t="s">
-        <v>52</v>
-      </c>
-      <c r="E13" t="s">
-        <v>52</v>
-      </c>
-      <c r="F13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J13" t="s">
-        <v>47</v>
-      </c>
-      <c r="N13" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" t="s">
+        <v>45</v>
+      </c>
+      <c r="M15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
         <v>66</v>
       </c>
-      <c r="D14" t="s">
-        <v>51</v>
-      </c>
-      <c r="E14" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" t="s">
-        <v>31</v>
-      </c>
-      <c r="J14" t="s">
-        <v>47</v>
-      </c>
-      <c r="N14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="B16" t="s">
         <v>67</v>
       </c>
-      <c r="D15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E15" t="s">
-        <v>50</v>
-      </c>
-      <c r="F15" t="s">
-        <v>31</v>
-      </c>
-      <c r="J15" t="s">
-        <v>47</v>
-      </c>
-      <c r="N15" t="s">
-        <v>48</v>
+      <c r="D16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+      <c r="M17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" t="s">
+        <v>77</v>
+      </c>
+      <c r="M18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" t="s">
+        <v>78</v>
+      </c>
+      <c r="M19" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+      <c r="M20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" t="s">
+        <v>80</v>
+      </c>
+      <c r="M21" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" t="s">
+        <v>81</v>
+      </c>
+      <c r="M22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" t="s">
+        <v>82</v>
+      </c>
+      <c r="M23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" t="s">
+        <v>123</v>
+      </c>
+      <c r="I26" t="s">
+        <v>138</v>
+      </c>
+      <c r="M26" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" t="s">
+        <v>107</v>
+      </c>
+      <c r="D27" t="s">
+        <v>124</v>
+      </c>
+      <c r="I27" t="s">
+        <v>138</v>
+      </c>
+      <c r="M27" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" t="s">
+        <v>125</v>
+      </c>
+      <c r="I28" t="s">
+        <v>138</v>
+      </c>
+      <c r="M28" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" t="s">
+        <v>109</v>
+      </c>
+      <c r="D29" t="s">
+        <v>126</v>
+      </c>
+      <c r="I29" t="s">
+        <v>139</v>
+      </c>
+      <c r="M29" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>103</v>
+      </c>
+      <c r="B30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" t="s">
+        <v>127</v>
+      </c>
+      <c r="I30" t="s">
+        <v>139</v>
+      </c>
+      <c r="M30" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>103</v>
+      </c>
+      <c r="B31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" t="s">
+        <v>128</v>
+      </c>
+      <c r="I31" t="s">
+        <v>139</v>
+      </c>
+      <c r="M31" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>103</v>
+      </c>
+      <c r="B32" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" t="s">
+        <v>112</v>
+      </c>
+      <c r="D32" t="s">
+        <v>129</v>
+      </c>
+      <c r="I32" t="s">
+        <v>139</v>
+      </c>
+      <c r="M32" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" t="s">
+        <v>113</v>
+      </c>
+      <c r="D33" t="s">
+        <v>130</v>
+      </c>
+      <c r="I33" t="s">
+        <v>139</v>
+      </c>
+      <c r="M33" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" t="s">
+        <v>96</v>
+      </c>
+      <c r="C34" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" t="s">
+        <v>131</v>
+      </c>
+      <c r="I34" t="s">
+        <v>139</v>
+      </c>
+      <c r="M34" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" t="s">
+        <v>115</v>
+      </c>
+      <c r="D35" t="s">
+        <v>132</v>
+      </c>
+      <c r="I35" t="s">
+        <v>139</v>
+      </c>
+      <c r="M35" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>103</v>
+      </c>
+      <c r="B36" t="s">
+        <v>98</v>
+      </c>
+      <c r="C36" t="s">
+        <v>116</v>
+      </c>
+      <c r="D36" t="s">
+        <v>133</v>
+      </c>
+      <c r="I36" t="s">
+        <v>140</v>
+      </c>
+      <c r="M36" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37" t="s">
+        <v>117</v>
+      </c>
+      <c r="D37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I37" t="s">
+        <v>138</v>
+      </c>
+      <c r="M37" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>103</v>
+      </c>
+      <c r="B38" t="s">
+        <v>100</v>
+      </c>
+      <c r="C38" t="s">
+        <v>118</v>
+      </c>
+      <c r="D38" t="s">
+        <v>135</v>
+      </c>
+      <c r="I38" t="s">
+        <v>141</v>
+      </c>
+      <c r="M38" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>103</v>
+      </c>
+      <c r="B39" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" t="s">
+        <v>119</v>
+      </c>
+      <c r="D39" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" t="s">
+        <v>120</v>
+      </c>
+      <c r="D40" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>149</v>
+      </c>
+      <c r="B41" t="s">
+        <v>150</v>
+      </c>
+      <c r="C41" t="s">
+        <v>151</v>
+      </c>
+      <c r="D41" t="s">
+        <v>152</v>
+      </c>
+      <c r="M41" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>149</v>
+      </c>
+      <c r="B42" t="s">
+        <v>153</v>
+      </c>
+      <c r="C42" t="s">
+        <v>154</v>
+      </c>
+      <c r="D42" t="s">
+        <v>155</v>
+      </c>
+      <c r="M42" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>149</v>
+      </c>
+      <c r="B43" t="s">
+        <v>156</v>
+      </c>
+      <c r="C43" t="s">
+        <v>157</v>
+      </c>
+      <c r="D43" t="s">
+        <v>158</v>
+      </c>
+      <c r="M43" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>149</v>
+      </c>
+      <c r="B44" t="s">
+        <v>159</v>
+      </c>
+      <c r="C44" t="s">
+        <v>160</v>
+      </c>
+      <c r="D44" t="s">
+        <v>161</v>
+      </c>
+      <c r="M44" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
+        <v>149</v>
+      </c>
+      <c r="B45" t="s">
+        <v>162</v>
+      </c>
+      <c r="C45" t="s">
+        <v>163</v>
+      </c>
+      <c r="D45" t="s">
+        <v>164</v>
+      </c>
+      <c r="M45" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>149</v>
+      </c>
+      <c r="B46" t="s">
+        <v>165</v>
+      </c>
+      <c r="C46" t="s">
+        <v>166</v>
+      </c>
+      <c r="D46" t="s">
+        <v>167</v>
+      </c>
+      <c r="M46" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>149</v>
+      </c>
+      <c r="B47" t="s">
+        <v>168</v>
+      </c>
+      <c r="C47" t="s">
+        <v>169</v>
+      </c>
+      <c r="D47" t="s">
+        <v>170</v>
+      </c>
+      <c r="M47" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD15" xr:uid="{B4F619F0-927D-42BE-B802-34E76A1D5A02}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD15">
-      <sortCondition ref="B1:B15"/>
+  <autoFilter ref="A1:AC15" xr:uid="{B4F619F0-927D-42BE-B802-34E76A1D5A02}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC15">
+      <sortCondition ref="A1:A15"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="18" type="noConversion"/>

</xml_diff>

<commit_message>
Added context-aware prestep section context
</commit_message>
<xml_diff>
--- a/CDE_ID_detective_revamp/in/Testfile.xlsx
+++ b/CDE_ID_detective_revamp/in/Testfile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmaefos\Code Stuffs\CDE_detective\CDE_ID_detective_revamp\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817B149D-0F69-43F3-8A18-7056A50B2854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A64F1D-8F3C-4056-850A-EC6EC69AC4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19305" yWindow="4500" windowWidth="19410" windowHeight="20985" xr2:uid="{B4172F7E-1829-43FF-A6F3-7109D1C548C2}"/>
+    <workbookView xWindow="-36585" yWindow="7755" windowWidth="25830" windowHeight="15105" xr2:uid="{B4172F7E-1829-43FF-A6F3-7109D1C548C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1421,8 +1421,35 @@
   <dimension ref="A1:AC47"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="33.19921875" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="1" max="1" width="30.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.9296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.06640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.46484375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.86328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="32.3984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="35.73046875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="33.3984375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="31.796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.265625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="30.53125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="26.59765625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.73046875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.73046875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="24.06640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="20.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.45">

</xml_diff>